<commit_message>
Actualizar datos 2026 (2026-04-13)
</commit_message>
<xml_diff>
--- a/data/asistencia/Caliente 2026.xlsx
+++ b/data/asistencia/Caliente 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="41">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,31 +82,31 @@
     <t>-</t>
   </si>
   <si>
-    <t>41.18%</t>
+    <t>97.72%</t>
   </si>
   <si>
     <t>Lateral</t>
   </si>
   <si>
-    <t>1.70%</t>
+    <t>6.09%</t>
   </si>
   <si>
     <t>Lateral Preferente</t>
   </si>
   <si>
-    <t>21.32%</t>
+    <t>50.05%</t>
   </si>
   <si>
     <t>Palco Bronce 1ra</t>
   </si>
   <si>
-    <t>0.00%</t>
+    <t>30.95%</t>
   </si>
   <si>
     <t>Palco Bronce 3ra</t>
   </si>
   <si>
-    <t>17.95%</t>
+    <t>55.13%</t>
   </si>
   <si>
     <t>Palco Oro</t>
@@ -118,13 +118,13 @@
     <t>Palco Plata 1ra</t>
   </si>
   <si>
-    <t>30.00%</t>
+    <t>98.33%</t>
   </si>
   <si>
     <t>Palco Plata 3ra</t>
   </si>
   <si>
-    <t>94.44%</t>
+    <t>96.30%</t>
   </si>
   <si>
     <t>Palco Platino</t>
@@ -133,7 +133,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>19.23%</t>
+    <t>43.42%</t>
   </si>
 </sst>
 </file>
@@ -646,13 +646,13 @@
         <v>1887</v>
       </c>
       <c r="C6" s="6">
-        <v>151</v>
+        <v>1202</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="6">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
@@ -670,7 +670,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="6">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="L6" s="6">
         <v>16</v>
@@ -679,16 +679,16 @@
         <v>22</v>
       </c>
       <c r="N6" s="6">
-        <v>225</v>
-      </c>
-      <c r="O6" s="6">
-        <v>38</v>
+        <v>266</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>777</v>
+        <v>1844</v>
       </c>
       <c r="Q6" s="6">
-        <v>1110</v>
+        <v>43</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -701,8 +701,8 @@
       <c r="B7" s="6">
         <v>3300</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>22</v>
+      <c r="C7" s="6">
+        <v>120</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -726,7 +726,7 @@
         <v>22</v>
       </c>
       <c r="K7" s="6">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L7" s="6">
         <v>3</v>
@@ -735,16 +735,16 @@
         <v>22</v>
       </c>
       <c r="N7" s="6">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P7" s="6">
-        <v>56</v>
+        <v>201</v>
       </c>
       <c r="Q7" s="6">
-        <v>3244</v>
+        <v>3099</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -758,7 +758,7 @@
         <v>1027</v>
       </c>
       <c r="C8" s="6">
-        <v>7</v>
+        <v>219</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>22</v>
@@ -782,7 +782,7 @@
         <v>22</v>
       </c>
       <c r="K8" s="6">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L8" s="6">
         <v>1</v>
@@ -791,16 +791,16 @@
         <v>22</v>
       </c>
       <c r="N8" s="6">
-        <v>200</v>
-      </c>
-      <c r="O8" s="6">
-        <v>1</v>
+        <v>280</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P8" s="6">
-        <v>219</v>
+        <v>514</v>
       </c>
       <c r="Q8" s="6">
-        <v>808</v>
+        <v>513</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>27</v>
@@ -813,8 +813,8 @@
       <c r="B9" s="6">
         <v>84</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>22</v>
+      <c r="C9" s="6">
+        <v>26</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>22</v>
@@ -852,11 +852,11 @@
       <c r="O9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P9" s="6" t="s">
-        <v>22</v>
+      <c r="P9" s="6">
+        <v>26</v>
       </c>
       <c r="Q9" s="6">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -869,8 +869,8 @@
       <c r="B10" s="6">
         <v>78</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
+      <c r="C10" s="6">
+        <v>24</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>22</v>
@@ -894,7 +894,7 @@
         <v>22</v>
       </c>
       <c r="K10" s="6">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>22</v>
@@ -909,10 +909,10 @@
         <v>22</v>
       </c>
       <c r="P10" s="6">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="Q10" s="6">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="R10" s="6" t="s">
         <v>31</v>
@@ -981,8 +981,8 @@
       <c r="B12" s="6">
         <v>60</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>22</v>
+      <c r="C12" s="6">
+        <v>41</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
@@ -1021,10 +1021,10 @@
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="Q12" s="6">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
@@ -1037,8 +1037,8 @@
       <c r="B13" s="6">
         <v>54</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>22</v>
+      <c r="C13" s="6">
+        <v>7</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
@@ -1073,14 +1073,14 @@
       <c r="N13" s="6">
         <v>12</v>
       </c>
-      <c r="O13" s="6">
-        <v>6</v>
+      <c r="O13" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q13" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>